<commit_message>
Update embedded IG with validated ConceptMaps and fixed codes
Rebuilt after fixing 105 validation errors (canonical URL, fabricated
codes, display names, interpretation version tracking). Down to 17
errors (5 unfixable R4/R4B dependency mismatches + 12 ConceptMap
URL fixes pending next rebuild).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/bw_amr_ig/CodeSystem-botswana-amr-local-method-cs.xlsx
+++ b/static/bw_amr_ig/CodeSystem-botswana-amr-local-method-cs.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://bw.health.gov/fhir/ImplementationGuide/bw-amr-ig/CodeSystem/botswana-amr-local-method-cs</t>
+    <t>http://bw.health.gov/fhir/amr/CodeSystem/botswana-amr-local-method-cs</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-13T15:54:56-04:00</t>
+    <t>2026-03-13T21:27:21-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>